<commit_message>
Lowered max player speed to 350 until player clip through walls problem is fixed. Moved objects rendering under particles. Resized sword enemy sprite.
</commit_message>
<xml_diff>
--- a/doc/bug-report.xlsx
+++ b/doc/bug-report.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="207">
   <si>
     <t>#</t>
   </si>
@@ -528,6 +528,9 @@
     <t>Observe 3 merged bee enemies in bee room.</t>
   </si>
   <si>
+    <t>Set a max bullet size instead so that this situation does not happen.</t>
+  </si>
+  <si>
     <t>Most enemies are pretty centered, so manual offsets defined per enemt should be fine for now.</t>
   </si>
   <si>
@@ -621,7 +624,7 @@
     <t>33 - Push console replacing bullets</t>
   </si>
   <si>
-    <t>Occasionally, the push console replaces the latest bullet on the stack instead of giving a new one.</t>
+    <t>Occasionally, the push console replaces the latest bullet on the stack instead of giving a new one. NOTE: need to assess reproduceability to determine if bug is actually there.</t>
   </si>
   <si>
     <t>The push console should only add new bullets.</t>
@@ -13915,9 +13918,11 @@
         <v>43</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="F3" s="5"/>
+        <v>12</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>32</v>
+      </c>
       <c r="G3" s="2" t="s">
         <v>86</v>
       </c>
@@ -13925,7 +13930,7 @@
         <v>87</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>88</v>
+        <v>171</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>89</v>
@@ -13957,7 +13962,7 @@
         <v>133</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>135</v>
@@ -13977,9 +13982,11 @@
         <v>19</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="F5" s="5"/>
+        <v>12</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>20</v>
+      </c>
       <c r="G5" s="2" t="s">
         <v>137</v>
       </c>
@@ -14045,13 +14052,13 @@
         <v>20</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>160</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>162</v>
@@ -14122,7 +14129,7 @@
         <v>12</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>168</v>
@@ -14139,7 +14146,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B10" s="3">
         <v>45607.0</v>
@@ -14157,16 +14164,16 @@
         <v>20</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="K10" s="5"/>
       <c r="L10" s="5"/>
@@ -14187,7 +14194,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B11" s="3">
         <v>45607.0</v>
@@ -14205,16 +14212,16 @@
         <v>20</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="K11" s="5"/>
       <c r="L11" s="5"/>
@@ -14235,7 +14242,7 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B12" s="3">
         <v>45610.0</v>
@@ -14250,19 +14257,19 @@
         <v>12</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K12" s="5"/>
       <c r="L12" s="5"/>
@@ -14283,7 +14290,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B13" s="8">
         <v>45613.0</v>
@@ -14301,21 +14308,21 @@
         <v>32</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B14" s="3">
         <v>45613.0</v>
@@ -14331,16 +14338,16 @@
       </c>
       <c r="F14" s="5"/>
       <c r="G14" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="K14" s="5"/>
       <c r="L14" s="5"/>
@@ -14361,7 +14368,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B15" s="3">
         <v>45613.0</v>
@@ -14377,16 +14384,16 @@
       </c>
       <c r="F15" s="5"/>
       <c r="G15" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="K15" s="5"/>
       <c r="L15" s="5"/>
@@ -14405,12 +14412,18 @@
       <c r="Y15" s="5"/>
       <c r="Z15" s="5"/>
     </row>
+    <row r="16">
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E15">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E16">
       <formula1>"Resolved,Open ,Won't Fix"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D15">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D16">
       <formula1>"P0,P1,P2,P3,P4,P5"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>